<commit_message>
Added a bunch of files for graphs
</commit_message>
<xml_diff>
--- a/failure-data-set2/Chosen_Failure_Set.xlsx
+++ b/failure-data-set2/Chosen_Failure_Set.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rainb\University_Stuff\SENG438\Assignment 5\seng438-assignment-5\failure-data-set2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{272D7776-6BB7-41B5-8A89-9A7594E57404}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D4DAC54-F3D3-4CC7-951E-E942ACF12F00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -83,12 +83,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -393,10 +392,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -413,1174 +412,1110 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
         <v>0.14555555555555555</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2">
         <v>0.14555555555555549</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2">
         <v>0.14555555555555549</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2">
         <v>7.2777777777777775E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>0.22638888888888889</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3">
         <v>5</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3">
         <v>0.22638888888888889</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3">
         <v>8.0833333333333326E-2</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3">
         <v>4.0416666666666663E-2</v>
       </c>
-      <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>0.31055555555555553</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4">
         <v>4</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4">
         <v>0.31055555555555547</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4">
         <v>8.4166666666666667E-2</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4">
         <v>4.2083333333333327E-2</v>
       </c>
-      <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>0.47888888888888886</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5">
         <v>4</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5">
         <v>0.47888888888888892</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5">
         <v>0.16833333333333331</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5">
         <v>8.4166666666666667E-2</v>
       </c>
-      <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>0.79305555555555551</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6">
         <v>3</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6">
         <v>0.79305555555555551</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6">
         <v>0.31416666666666659</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6">
         <v>0.1570833333333333</v>
       </c>
-      <c r="J6" s="2"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
         <v>0.86861111111111111</v>
       </c>
-      <c r="B7" s="2">
-        <v>2</v>
-      </c>
-      <c r="C7" s="2">
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7">
         <v>0.86861111111111111</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7">
         <v>7.5555555555555556E-2</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7">
         <v>3.7777777777777778E-2</v>
       </c>
-      <c r="J7" s="2"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
         <v>1.0791666666666666</v>
       </c>
-      <c r="B8" s="2">
-        <v>2</v>
-      </c>
-      <c r="C8" s="2">
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8">
         <v>1.0791666666666671</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8">
         <v>0.21055555555555561</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8">
         <v>0.1052777777777778</v>
       </c>
-      <c r="J8" s="2"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
         <v>1.2605555555555557</v>
       </c>
-      <c r="B9" s="2">
-        <v>2</v>
-      </c>
-      <c r="C9" s="2">
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9">
         <v>1.2605555555555561</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9">
         <v>0.18138888888888891</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9">
         <v>9.0694444444444439E-2</v>
       </c>
-      <c r="J9" s="2"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
         <v>1.2961111111111112</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10">
         <v>1</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10">
         <v>1.296111111111111</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10">
         <v>3.5555555555555562E-2</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10">
         <v>1.7777777777777781E-2</v>
       </c>
-      <c r="J10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11">
         <v>1.3477777777777777</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11">
         <v>1</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11">
         <v>1.347777777777778</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11">
         <v>5.1666666666666673E-2</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11">
         <v>2.583333333333333E-2</v>
       </c>
-      <c r="J11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
         <v>1.3833333333333333</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12">
         <v>1</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12">
         <v>1.3833333333333331</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12">
         <v>3.5555555555555562E-2</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12">
         <v>1.7777777777777781E-2</v>
       </c>
-      <c r="J12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
         <v>1.7705555555555557</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13">
         <v>5</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13">
         <v>1.7705555555555561</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13">
         <v>0.38722222222222219</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13">
         <v>0.19361111111111109</v>
       </c>
-      <c r="J13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
         <v>1.9130555555555555</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14">
         <v>4</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14">
         <v>1.913055555555556</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14">
         <v>0.14249999999999999</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14">
         <v>7.1249999999999994E-2</v>
       </c>
-      <c r="J14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
         <v>2.2697222222222222</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15">
         <v>3</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15">
         <v>2.2697222222222222</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15">
         <v>0.35666666666666669</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15">
         <v>0.17833333333333329</v>
       </c>
-      <c r="J15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
         <v>2.4802777777777778</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16">
         <v>1</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16">
         <v>2.4802777777777778</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16">
         <v>0.21055555555555561</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16">
         <v>0.1052777777777778</v>
       </c>
-      <c r="J16" s="2"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
         <v>3.0602777777777779</v>
       </c>
-      <c r="B17" s="2">
-        <v>2</v>
-      </c>
-      <c r="C17" s="2">
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17">
         <v>3.0602777777777779</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17">
         <v>0.57999999999999996</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17">
         <v>0.28999999999999998</v>
       </c>
-      <c r="J17" s="2"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18">
         <v>3.1013888888888888</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18">
         <v>4</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18">
         <v>3.1013888888888892</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18">
         <v>4.1111111111111112E-2</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18">
         <v>2.055555555555556E-2</v>
       </c>
-      <c r="J18" s="2"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
         <v>3.1855555555555557</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19">
         <v>5</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19">
         <v>3.1855555555555561</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19">
         <v>8.4166666666666667E-2</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19">
         <v>4.2083333333333327E-2</v>
       </c>
-      <c r="J19" s="2"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20">
         <v>3.3666666666666667</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20">
         <v>4</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20">
         <v>3.3666666666666671</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20">
         <v>0.18111111111111111</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20">
         <v>9.0555555555555556E-2</v>
       </c>
-      <c r="J20" s="2"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>3.5966666666666667</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21">
         <v>3</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21">
         <v>3.5966666666666671</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21">
         <v>0.23</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21">
         <v>0.115</v>
       </c>
-      <c r="J21" s="2"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="2">
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22">
         <v>3.7294444444444443</v>
       </c>
-      <c r="B22" s="2">
-        <v>2</v>
-      </c>
-      <c r="C22" s="2">
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22">
         <v>3.7294444444444439</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22">
         <v>0.1327777777777778</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22">
         <v>6.6388888888888886E-2</v>
       </c>
-      <c r="J22" s="2"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="2">
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23">
         <v>4.4072222222222219</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23">
         <v>1</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C23">
         <v>4.4072222222222219</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23">
         <v>0.67777777777777781</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23">
         <v>0.33888888888888891</v>
       </c>
-      <c r="J23" s="2"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="2">
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24">
         <v>4.54</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24">
         <v>1</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C24">
         <v>4.54</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D24">
         <v>0.1327777777777778</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24">
         <v>6.6388888888888886E-2</v>
       </c>
-      <c r="J24" s="2"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="2">
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25">
         <v>4.6433333333333335</v>
       </c>
-      <c r="B25" s="2">
+      <c r="B25">
         <v>1</v>
       </c>
-      <c r="C25" s="2">
+      <c r="C25">
         <v>4.6433333333333344</v>
       </c>
-      <c r="D25" s="2">
+      <c r="D25">
         <v>0.1033333333333333</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25">
         <v>5.1666666666666673E-2</v>
       </c>
-      <c r="J25" s="2"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="2">
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26">
         <v>4.7663888888888888</v>
       </c>
-      <c r="B26" s="2">
-        <v>2</v>
-      </c>
-      <c r="C26" s="2">
+      <c r="B26">
+        <v>2</v>
+      </c>
+      <c r="C26">
         <v>4.7663888888888888</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26">
         <v>0.1230555555555556</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26">
         <v>6.1527777777777778E-2</v>
       </c>
-      <c r="J26" s="2"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="2">
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27">
         <v>4.9288888888888893</v>
       </c>
-      <c r="B27" s="2">
-        <v>2</v>
-      </c>
-      <c r="C27" s="2">
+      <c r="B27">
+        <v>2</v>
+      </c>
+      <c r="C27">
         <v>4.9288888888888893</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27">
         <v>0.16250000000000001</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27">
         <v>8.1250000000000003E-2</v>
       </c>
-      <c r="J27" s="2"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="2">
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28">
         <v>5.0130555555555558</v>
       </c>
-      <c r="B28" s="2">
+      <c r="B28">
         <v>4</v>
       </c>
-      <c r="C28" s="2">
+      <c r="C28">
         <v>5.0130555555555558</v>
       </c>
-      <c r="D28" s="2">
+      <c r="D28">
         <v>8.4166666666666667E-2</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28">
         <v>4.2083333333333327E-2</v>
       </c>
-      <c r="J28" s="2"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="2">
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29">
         <v>5.1233333333333331</v>
       </c>
-      <c r="B29" s="2">
+      <c r="B29">
         <v>5</v>
       </c>
-      <c r="C29" s="2">
+      <c r="C29">
         <v>5.1233333333333331</v>
       </c>
-      <c r="D29" s="2">
+      <c r="D29">
         <v>0.11027777777777779</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29">
         <v>5.513888888888889E-2</v>
       </c>
-      <c r="J29" s="2"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="2">
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30">
         <v>5.2819444444444441</v>
       </c>
-      <c r="B30" s="2">
+      <c r="B30">
         <v>4</v>
       </c>
-      <c r="C30" s="2">
+      <c r="C30">
         <v>5.2819444444444441</v>
       </c>
-      <c r="D30" s="2">
+      <c r="D30">
         <v>0.15861111111111109</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E30">
         <v>7.930555555555556E-2</v>
       </c>
-      <c r="J30" s="2"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="2">
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31">
         <v>5.4683333333333337</v>
       </c>
-      <c r="B31" s="2">
+      <c r="B31">
         <v>1</v>
       </c>
-      <c r="C31" s="2">
+      <c r="C31">
         <v>5.4683333333333337</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D31">
         <v>0.18638888888888891</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31">
         <v>9.3194444444444441E-2</v>
       </c>
-      <c r="J31" s="2"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="2">
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32">
         <v>5.5525000000000002</v>
       </c>
-      <c r="B32" s="2">
-        <v>2</v>
-      </c>
-      <c r="C32" s="2">
+      <c r="B32">
+        <v>2</v>
+      </c>
+      <c r="C32">
         <v>5.5525000000000002</v>
       </c>
-      <c r="D32" s="2">
+      <c r="D32">
         <v>8.4166666666666667E-2</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32">
         <v>4.2083333333333327E-2</v>
       </c>
-      <c r="J32" s="2"/>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" s="2">
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33">
         <v>5.9474999999999998</v>
       </c>
-      <c r="B33" s="2">
-        <v>2</v>
-      </c>
-      <c r="C33" s="2">
+      <c r="B33">
+        <v>2</v>
+      </c>
+      <c r="C33">
         <v>5.9474999999999998</v>
       </c>
-      <c r="D33" s="2">
+      <c r="D33">
         <v>0.39500000000000002</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33">
         <v>0.19750000000000001</v>
       </c>
-      <c r="J33" s="2"/>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="2">
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34">
         <v>6.1969444444444441</v>
       </c>
-      <c r="B34" s="2">
+      <c r="B34">
         <v>3</v>
       </c>
-      <c r="C34" s="2">
+      <c r="C34">
         <v>6.1969444444444441</v>
       </c>
-      <c r="D34" s="2">
+      <c r="D34">
         <v>0.24944444444444441</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34">
         <v>0.12472222222222221</v>
       </c>
-      <c r="J34" s="2"/>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" s="2">
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35">
         <v>6.2616666666666667</v>
       </c>
-      <c r="B35" s="2">
+      <c r="B35">
         <v>4</v>
       </c>
-      <c r="C35" s="2">
+      <c r="C35">
         <v>6.2616666666666667</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35">
         <v>6.4722222222222223E-2</v>
       </c>
-      <c r="E35" s="2">
+      <c r="E35">
         <v>3.2361111111111111E-2</v>
       </c>
-      <c r="J35" s="2"/>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="2">
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36">
         <v>6.7538888888888886</v>
       </c>
-      <c r="B36" s="2">
+      <c r="B36">
         <v>5</v>
       </c>
-      <c r="C36" s="2">
+      <c r="C36">
         <v>6.7538888888888886</v>
       </c>
-      <c r="D36" s="2">
+      <c r="D36">
         <v>0.49222222222222223</v>
       </c>
-      <c r="E36" s="2">
+      <c r="E36">
         <v>0.24611111111111111</v>
       </c>
-      <c r="J36" s="2"/>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" s="2">
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37">
         <v>7.2405555555555559</v>
       </c>
-      <c r="B37" s="2">
+      <c r="B37">
         <v>4</v>
       </c>
-      <c r="C37" s="2">
+      <c r="C37">
         <v>7.2405555555555559</v>
       </c>
-      <c r="D37" s="2">
+      <c r="D37">
         <v>0.48666666666666669</v>
       </c>
-      <c r="E37" s="2">
+      <c r="E37">
         <v>0.24333333333333329</v>
       </c>
-      <c r="J37" s="2"/>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38" s="2">
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38">
         <v>7.3311111111111114</v>
       </c>
-      <c r="B38" s="2">
-        <v>2</v>
-      </c>
-      <c r="C38" s="2">
+      <c r="B38">
+        <v>2</v>
+      </c>
+      <c r="C38">
         <v>7.3311111111111114</v>
       </c>
-      <c r="D38" s="2">
+      <c r="D38">
         <v>9.0555555555555556E-2</v>
       </c>
-      <c r="E38" s="2">
+      <c r="E38">
         <v>4.5277777777777778E-2</v>
       </c>
-      <c r="J38" s="2"/>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39" s="2">
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39">
         <v>7.5966666666666667</v>
       </c>
-      <c r="B39" s="2">
-        <v>2</v>
-      </c>
-      <c r="C39" s="2">
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39">
         <v>7.5966666666666667</v>
       </c>
-      <c r="D39" s="2">
+      <c r="D39">
         <v>0.26555555555555549</v>
       </c>
-      <c r="E39" s="2">
+      <c r="E39">
         <v>0.1327777777777778</v>
       </c>
-      <c r="J39" s="2"/>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A40" s="2">
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40">
         <v>7.7844444444444445</v>
       </c>
-      <c r="B40" s="2">
+      <c r="B40">
         <v>1</v>
       </c>
-      <c r="C40" s="2">
+      <c r="C40">
         <v>7.7844444444444436</v>
       </c>
-      <c r="D40" s="2">
+      <c r="D40">
         <v>0.18777777777777779</v>
       </c>
-      <c r="E40" s="2">
+      <c r="E40">
         <v>9.3888888888888883E-2</v>
       </c>
-      <c r="J40" s="2"/>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="2">
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41">
         <v>8.586666666666666</v>
       </c>
-      <c r="B41" s="2">
+      <c r="B41">
         <v>4</v>
       </c>
-      <c r="C41" s="2">
+      <c r="C41">
         <v>8.586666666666666</v>
       </c>
-      <c r="D41" s="2">
+      <c r="D41">
         <v>0.80222222222222217</v>
       </c>
-      <c r="E41" s="2">
+      <c r="E41">
         <v>0.40111111111111108</v>
       </c>
-      <c r="J41" s="2"/>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="2">
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42">
         <v>8.588055555555556</v>
       </c>
-      <c r="B42" s="2">
+      <c r="B42">
         <v>3</v>
       </c>
-      <c r="C42" s="2">
+      <c r="C42">
         <v>8.588055555555556</v>
       </c>
-      <c r="D42" s="2">
+      <c r="D42">
         <v>1.3888888888888889E-3</v>
       </c>
-      <c r="E42" s="2">
+      <c r="E42">
         <v>6.9444444444444447E-4</v>
       </c>
-      <c r="J42" s="2"/>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" s="2">
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43">
         <v>8.6333333333333329</v>
       </c>
-      <c r="B43" s="2">
+      <c r="B43">
         <v>3</v>
       </c>
-      <c r="C43" s="2">
+      <c r="C43">
         <v>8.6333333333333329</v>
       </c>
-      <c r="D43" s="2">
+      <c r="D43">
         <v>4.5277777777777778E-2</v>
       </c>
-      <c r="E43" s="2">
+      <c r="E43">
         <v>2.2638888888888889E-2</v>
       </c>
-      <c r="J43" s="2"/>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A44" s="2">
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44">
         <v>8.9474999999999998</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44">
         <v>4</v>
       </c>
-      <c r="C44" s="2">
+      <c r="C44">
         <v>8.9474999999999998</v>
       </c>
-      <c r="D44" s="2">
+      <c r="D44">
         <v>0.31416666666666659</v>
       </c>
-      <c r="E44" s="2">
+      <c r="E44">
         <v>0.1570833333333333</v>
       </c>
-      <c r="J44" s="2"/>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A45" s="2">
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45">
         <v>9.6894444444444439</v>
       </c>
-      <c r="B45" s="2">
+      <c r="B45">
         <v>3</v>
       </c>
-      <c r="C45" s="2">
+      <c r="C45">
         <v>9.6894444444444439</v>
       </c>
-      <c r="D45" s="2">
+      <c r="D45">
         <v>0.74194444444444441</v>
       </c>
-      <c r="E45" s="2">
+      <c r="E45">
         <v>0.3709722222222222</v>
       </c>
-      <c r="J45" s="2"/>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A46" s="2">
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46">
         <v>9.8291666666666675</v>
       </c>
-      <c r="B46" s="2">
+      <c r="B46">
         <v>3</v>
       </c>
-      <c r="C46" s="2">
+      <c r="C46">
         <v>9.8291666666666675</v>
       </c>
-      <c r="D46" s="2">
+      <c r="D46">
         <v>0.13972222222222219</v>
       </c>
-      <c r="E46" s="2">
+      <c r="E46">
         <v>6.986111111111111E-2</v>
       </c>
-      <c r="J46" s="2"/>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A47" s="2">
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47">
         <v>10.000833333333333</v>
       </c>
-      <c r="B47" s="2">
+      <c r="B47">
         <v>4</v>
       </c>
-      <c r="C47" s="2">
+      <c r="C47">
         <v>10.000833333333331</v>
       </c>
-      <c r="D47" s="2">
+      <c r="D47">
         <v>0.17166666666666669</v>
       </c>
-      <c r="E47" s="2">
+      <c r="E47">
         <v>8.5833333333333331E-2</v>
       </c>
-      <c r="J47" s="2"/>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A48" s="2">
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48">
         <v>10.340833333333334</v>
       </c>
-      <c r="B48" s="2">
+      <c r="B48">
         <v>1</v>
       </c>
-      <c r="C48" s="2">
+      <c r="C48">
         <v>10.340833333333331</v>
       </c>
-      <c r="D48" s="2">
+      <c r="D48">
         <v>0.34</v>
       </c>
-      <c r="E48" s="2">
+      <c r="E48">
         <v>0.17</v>
       </c>
-      <c r="J48" s="2"/>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A49" s="2">
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49">
         <v>10.473611111111111</v>
       </c>
-      <c r="B49" s="2">
+      <c r="B49">
         <v>5</v>
       </c>
-      <c r="C49" s="2">
+      <c r="C49">
         <v>10.47361111111111</v>
       </c>
-      <c r="D49" s="2">
+      <c r="D49">
         <v>0.1327777777777778</v>
       </c>
-      <c r="E49" s="2">
+      <c r="E49">
         <v>6.6388888888888886E-2</v>
       </c>
-      <c r="J49" s="2"/>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" s="2">
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50">
         <v>10.755277777777778</v>
       </c>
-      <c r="B50" s="2">
+      <c r="B50">
         <v>1</v>
       </c>
-      <c r="C50" s="2">
+      <c r="C50">
         <v>10.755277777777779</v>
       </c>
-      <c r="D50" s="2">
+      <c r="D50">
         <v>0.28166666666666668</v>
       </c>
-      <c r="E50" s="2">
+      <c r="E50">
         <v>0.14083333333333331</v>
       </c>
-      <c r="J50" s="2"/>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A51" s="2">
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51">
         <v>12.111388888888889</v>
       </c>
-      <c r="B51" s="2">
+      <c r="B51">
         <v>5</v>
       </c>
-      <c r="C51" s="2">
+      <c r="C51">
         <v>12.111388888888889</v>
       </c>
-      <c r="D51" s="2">
+      <c r="D51">
         <v>1.356111111111111</v>
       </c>
-      <c r="E51" s="2">
+      <c r="E51">
         <v>0.67805555555555552</v>
       </c>
-      <c r="J51" s="2"/>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A52" s="2">
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52">
         <v>12.328333333333333</v>
       </c>
-      <c r="B52" s="2">
+      <c r="B52">
         <v>1</v>
       </c>
-      <c r="C52" s="2">
+      <c r="C52">
         <v>12.32833333333333</v>
       </c>
-      <c r="D52" s="2">
+      <c r="D52">
         <v>0.21694444444444441</v>
       </c>
-      <c r="E52" s="2">
+      <c r="E52">
         <v>0.10847222222222221</v>
       </c>
-      <c r="J52" s="2"/>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A53" s="2">
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53">
         <v>12.383333333333333</v>
       </c>
-      <c r="B53" s="2">
-        <v>2</v>
-      </c>
-      <c r="C53" s="2">
+      <c r="B53">
+        <v>2</v>
+      </c>
+      <c r="C53">
         <v>12.383333333333329</v>
       </c>
-      <c r="D53" s="2">
+      <c r="D53">
         <v>5.5E-2</v>
       </c>
-      <c r="E53" s="2">
+      <c r="E53">
         <v>2.75E-2</v>
       </c>
-      <c r="J53" s="2"/>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A54" s="2">
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54">
         <v>12.834722222222222</v>
       </c>
-      <c r="B54" s="2">
-        <v>2</v>
-      </c>
-      <c r="C54" s="2">
+      <c r="B54">
+        <v>2</v>
+      </c>
+      <c r="C54">
         <v>12.83472222222222</v>
       </c>
-      <c r="D54" s="2">
+      <c r="D54">
         <v>0.4513888888888889</v>
       </c>
-      <c r="E54" s="2">
+      <c r="E54">
         <v>0.22569444444444439</v>
       </c>
-      <c r="J54" s="2"/>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A55" s="2">
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55">
         <v>13.064722222222223</v>
       </c>
-      <c r="B55" s="2">
+      <c r="B55">
         <v>4</v>
       </c>
-      <c r="C55" s="2">
+      <c r="C55">
         <v>13.064722222222221</v>
       </c>
-      <c r="D55" s="2">
+      <c r="D55">
         <v>0.23</v>
       </c>
-      <c r="E55" s="2">
+      <c r="E55">
         <v>0.115</v>
       </c>
-      <c r="J55" s="2"/>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A56" s="2">
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56">
         <v>14.023333333333333</v>
       </c>
-      <c r="B56" s="2">
+      <c r="B56">
         <v>3</v>
       </c>
-      <c r="C56" s="2">
+      <c r="C56">
         <v>14.02333333333333</v>
       </c>
-      <c r="D56" s="2">
+      <c r="D56">
         <v>0.95861111111111108</v>
       </c>
-      <c r="E56" s="2">
+      <c r="E56">
         <v>0.47930555555555548</v>
       </c>
-      <c r="J56" s="2"/>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A57" s="2">
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57">
         <v>14.66611111111111</v>
       </c>
-      <c r="B57" s="2">
-        <v>2</v>
-      </c>
-      <c r="C57" s="2">
+      <c r="B57">
+        <v>2</v>
+      </c>
+      <c r="C57">
         <v>14.66611111111111</v>
       </c>
-      <c r="D57" s="2">
+      <c r="D57">
         <v>0.64277777777777778</v>
       </c>
-      <c r="E57" s="2">
+      <c r="E57">
         <v>0.32138888888888889</v>
       </c>
-      <c r="J57" s="2"/>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A58" s="2">
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58">
         <v>14.934722222222222</v>
       </c>
-      <c r="B58" s="2">
+      <c r="B58">
         <v>3</v>
       </c>
-      <c r="C58" s="2">
+      <c r="C58">
         <v>14.93472222222222</v>
       </c>
-      <c r="D58" s="2">
+      <c r="D58">
         <v>0.26861111111111108</v>
       </c>
-      <c r="E58" s="2">
+      <c r="E58">
         <v>0.13430555555555559</v>
       </c>
-      <c r="J58" s="2"/>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A59" s="2">
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59">
         <v>15.553888888888888</v>
       </c>
-      <c r="B59" s="2">
+      <c r="B59">
         <v>4</v>
       </c>
-      <c r="C59" s="2">
+      <c r="C59">
         <v>15.55388888888889</v>
       </c>
-      <c r="D59" s="2">
+      <c r="D59">
         <v>0.61916666666666664</v>
       </c>
-      <c r="E59" s="2">
+      <c r="E59">
         <v>0.30958333333333332</v>
       </c>
-      <c r="J59" s="2"/>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A60" s="2">
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60">
         <v>16.003888888888888</v>
       </c>
-      <c r="B60" s="2">
+      <c r="B60">
         <v>5</v>
       </c>
-      <c r="C60" s="2">
+      <c r="C60">
         <v>16.003888888888891</v>
       </c>
-      <c r="D60" s="2">
+      <c r="D60">
         <v>0.45</v>
       </c>
-      <c r="E60" s="2">
+      <c r="E60">
         <v>0.22500000000000001</v>
       </c>
-      <c r="J60" s="2"/>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A61" s="2">
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61">
         <v>16.173888888888889</v>
       </c>
-      <c r="B61" s="2">
+      <c r="B61">
         <v>5</v>
       </c>
-      <c r="C61" s="2">
+      <c r="C61">
         <v>16.173888888888889</v>
       </c>
-      <c r="D61" s="2">
+      <c r="D61">
         <v>0.17</v>
       </c>
-      <c r="E61" s="2">
+      <c r="E61">
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="J61" s="2"/>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A62" s="2">
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62">
         <v>16.322777777777777</v>
       </c>
-      <c r="B62" s="2">
+      <c r="B62">
         <v>1</v>
       </c>
-      <c r="C62" s="2">
+      <c r="C62">
         <v>16.32277777777778</v>
       </c>
-      <c r="D62" s="2">
+      <c r="D62">
         <v>0.1488888888888889</v>
       </c>
-      <c r="E62" s="2">
+      <c r="E62">
         <v>7.4444444444444438E-2</v>
       </c>
-      <c r="J62" s="2"/>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A63" s="2">
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63">
         <v>16.503055555555555</v>
       </c>
-      <c r="B63" s="2">
-        <v>2</v>
-      </c>
-      <c r="C63" s="2">
+      <c r="B63">
+        <v>2</v>
+      </c>
+      <c r="C63">
         <v>16.503055555555559</v>
       </c>
-      <c r="D63" s="2">
+      <c r="D63">
         <v>0.18027777777777779</v>
       </c>
-      <c r="E63" s="2">
+      <c r="E63">
         <v>9.0138888888888893E-2</v>
       </c>
-      <c r="J63" s="2"/>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A64" s="2">
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64">
         <v>17.040555555555557</v>
       </c>
-      <c r="B64" s="2">
-        <v>2</v>
-      </c>
-      <c r="C64" s="2">
+      <c r="B64">
+        <v>2</v>
+      </c>
+      <c r="C64">
         <v>17.04055555555556</v>
       </c>
-      <c r="D64" s="2">
+      <c r="D64">
         <v>0.53749999999999998</v>
       </c>
-      <c r="E64" s="2">
+      <c r="E64">
         <v>0.26874999999999999</v>
       </c>
-      <c r="J64" s="2"/>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A65" s="2">
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65">
         <v>17.066388888888888</v>
       </c>
-      <c r="B65" s="2">
+      <c r="B65">
         <v>4</v>
       </c>
-      <c r="C65" s="2">
+      <c r="C65">
         <v>17.066388888888891</v>
       </c>
-      <c r="D65" s="2">
+      <c r="D65">
         <v>2.583333333333333E-2</v>
       </c>
-      <c r="E65" s="2">
+      <c r="E65">
         <v>1.291666666666667E-2</v>
       </c>
-      <c r="J65" s="2"/>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A66" s="2">
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66">
         <v>17.928333333333335</v>
       </c>
-      <c r="B66" s="2">
-        <v>2</v>
-      </c>
-      <c r="C66" s="2">
+      <c r="B66">
+        <v>2</v>
+      </c>
+      <c r="C66">
         <v>17.928333333333331</v>
       </c>
-      <c r="D66" s="2">
+      <c r="D66">
         <v>0.8619444444444444</v>
       </c>
-      <c r="E66" s="2">
+      <c r="E66">
         <v>0.4309722222222222</v>
       </c>
-      <c r="J66" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Finished the Laplace scores
</commit_message>
<xml_diff>
--- a/failure-data-set2/Chosen_Failure_Set.xlsx
+++ b/failure-data-set2/Chosen_Failure_Set.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rainb\University_Stuff\SENG438\Assignment 5\seng438-assignment-5\failure-data-set2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D4DAC54-F3D3-4CC7-951E-E942ACF12F00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC95E355-CD8D-445E-A0E1-54FD950D2CCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -392,10 +392,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E66"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L66"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -412,7 +412,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0.14555555555555555</v>
       </c>
@@ -428,8 +428,23 @@
       <c r="E2">
         <v>7.2777777777777775E-2</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H2">
+        <f>B2</f>
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <f>SUM(A2:A66)/SUM(B2:B66)</f>
+        <v>2.6081177899210681</v>
+      </c>
+      <c r="J2">
+        <v>0.145602068</v>
+      </c>
+      <c r="L2">
+        <f>(J$2-(A2/2))/(A2*SQRT(1/(12*H2)))</f>
+        <v>1.7331577652065233</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>0.22638888888888889</v>
       </c>
@@ -445,10 +460,18 @@
       <c r="E3">
         <v>4.0416666666666663E-2</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H3">
+        <f>H2+B3</f>
+        <v>6</v>
+      </c>
+      <c r="L3">
+        <f>(J$2-(A3/2))/(A3*SQRT(1/(12*H3)))</f>
+        <v>1.2146700568606705</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>0.31055555555555553</v>
+        <v>0.31055555555555597</v>
       </c>
       <c r="B4">
         <v>4</v>
@@ -462,8 +485,16 @@
       <c r="E4">
         <v>4.2083333333333327E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H4">
+        <f>H3+B4</f>
+        <v>10</v>
+      </c>
+      <c r="L4">
+        <f>(J$2-(A4/2))/(A4*SQRT(1/(12*H4)))</f>
+        <v>-0.34129832233603324</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>0.47888888888888886</v>
       </c>
@@ -479,8 +510,16 @@
       <c r="E5">
         <v>8.4166666666666667E-2</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H5">
+        <f>H4+B5</f>
+        <v>14</v>
+      </c>
+      <c r="L5">
+        <f t="shared" ref="L3:L66" si="0">(J$2-(A5/2))/(A5*SQRT(1/(12*H5)))</f>
+        <v>-2.5399132131458932</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>0.79305555555555551</v>
       </c>
@@ -496,8 +535,16 @@
       <c r="E6">
         <v>0.1570833333333333</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H6">
+        <f>H5+B6</f>
+        <v>17</v>
+      </c>
+      <c r="L6">
+        <f t="shared" si="0"/>
+        <v>-4.5191487146294449</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>0.86861111111111111</v>
       </c>
@@ -513,10 +560,18 @@
       <c r="E7">
         <v>3.7777777777777778E-2</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H7">
+        <f t="shared" ref="H4:H66" si="1">H6+B7</f>
+        <v>19</v>
+      </c>
+      <c r="L7">
+        <f t="shared" si="0"/>
+        <v>-5.018732788581322</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1.0791666666666666</v>
+        <v>1.0791666666666699</v>
       </c>
       <c r="B8">
         <v>2</v>
@@ -530,8 +585,16 @@
       <c r="E8">
         <v>0.1052777777777778</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H8">
+        <f t="shared" si="1"/>
+        <v>21</v>
+      </c>
+      <c r="L8">
+        <f t="shared" si="0"/>
+        <v>-5.7954520732756682</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1.2605555555555557</v>
       </c>
@@ -547,8 +610,16 @@
       <c r="E9">
         <v>9.0694444444444439E-2</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H9">
+        <f t="shared" si="1"/>
+        <v>23</v>
+      </c>
+      <c r="L9">
+        <f t="shared" si="0"/>
+        <v>-6.3876896164921284</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>1.2961111111111112</v>
       </c>
@@ -564,8 +635,16 @@
       <c r="E10">
         <v>1.7777777777777781E-2</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H10">
+        <f t="shared" si="1"/>
+        <v>24</v>
+      </c>
+      <c r="L10">
+        <f t="shared" si="0"/>
+        <v>-6.5788483453728768</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1.3477777777777777</v>
       </c>
@@ -581,8 +660,16 @@
       <c r="E11">
         <v>2.583333333333333E-2</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H11">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+      <c r="L11">
+        <f t="shared" si="0"/>
+        <v>-6.7890985430645943</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>1.3833333333333333</v>
       </c>
@@ -598,8 +685,16 @@
       <c r="E12">
         <v>1.7777777777777781E-2</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H12">
+        <f t="shared" si="1"/>
+        <v>26</v>
+      </c>
+      <c r="L12">
+        <f t="shared" si="0"/>
+        <v>-6.9725955946861999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1.7705555555555557</v>
       </c>
@@ -615,8 +710,16 @@
       <c r="E13">
         <v>0.19361111111111109</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H13">
+        <f t="shared" si="1"/>
+        <v>31</v>
+      </c>
+      <c r="L13">
+        <f t="shared" si="0"/>
+        <v>-8.0575548156106986</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>1.9130555555555555</v>
       </c>
@@ -632,8 +735,16 @@
       <c r="E14">
         <v>7.1249999999999994E-2</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H14">
+        <f t="shared" si="1"/>
+        <v>35</v>
+      </c>
+      <c r="L14">
+        <f t="shared" si="0"/>
+        <v>-8.6871662444017517</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2.2697222222222222</v>
       </c>
@@ -649,8 +760,16 @@
       <c r="E15">
         <v>0.17833333333333329</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H15">
+        <f t="shared" si="1"/>
+        <v>38</v>
+      </c>
+      <c r="L15">
+        <f t="shared" si="0"/>
+        <v>-9.3072148753829449</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2.4802777777777778</v>
       </c>
@@ -666,8 +785,16 @@
       <c r="E16">
         <v>0.1052777777777778</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H16">
+        <f t="shared" si="1"/>
+        <v>39</v>
+      </c>
+      <c r="L16">
+        <f t="shared" si="0"/>
+        <v>-9.5466935178543881</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>3.0602777777777779</v>
       </c>
@@ -683,8 +810,16 @@
       <c r="E17">
         <v>0.28999999999999998</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H17">
+        <f t="shared" si="1"/>
+        <v>41</v>
+      </c>
+      <c r="L17">
+        <f t="shared" si="0"/>
+        <v>-10.035204168744762</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>3.1013888888888888</v>
       </c>
@@ -700,8 +835,16 @@
       <c r="E18">
         <v>2.055555555555556E-2</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H18">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+      <c r="L18">
+        <f t="shared" si="0"/>
+        <v>-10.527991623395472</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>3.1855555555555557</v>
       </c>
@@ -717,8 +860,16 @@
       <c r="E19">
         <v>4.2083333333333327E-2</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H19">
+        <f t="shared" si="1"/>
+        <v>50</v>
+      </c>
+      <c r="L19">
+        <f t="shared" si="0"/>
+        <v>-11.127861358196959</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>3.3666666666666667</v>
       </c>
@@ -734,8 +885,16 @@
       <c r="E20">
         <v>9.0555555555555556E-2</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H20">
+        <f t="shared" si="1"/>
+        <v>54</v>
+      </c>
+      <c r="L20">
+        <f t="shared" si="0"/>
+        <v>-11.627004176124276</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>3.5966666666666667</v>
       </c>
@@ -751,8 +910,16 @@
       <c r="E21">
         <v>0.115</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="H21">
+        <f t="shared" si="1"/>
+        <v>57</v>
+      </c>
+      <c r="L21">
+        <f t="shared" si="0"/>
+        <v>-12.01794200143892</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>3.7294444444444443</v>
       </c>
@@ -769,7 +936,7 @@
         <v>6.6388888888888886E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>4.4072222222222219</v>
       </c>
@@ -786,7 +953,7 @@
         <v>0.33888888888888891</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>4.54</v>
       </c>
@@ -803,7 +970,7 @@
         <v>6.6388888888888886E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>4.6433333333333335</v>
       </c>
@@ -820,7 +987,7 @@
         <v>5.1666666666666673E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>4.7663888888888888</v>
       </c>
@@ -837,7 +1004,7 @@
         <v>6.1527777777777778E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>4.9288888888888893</v>
       </c>
@@ -854,7 +1021,7 @@
         <v>8.1250000000000003E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>5.0130555555555558</v>
       </c>
@@ -871,7 +1038,7 @@
         <v>4.2083333333333327E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>5.1233333333333331</v>
       </c>
@@ -888,7 +1055,7 @@
         <v>5.513888888888889E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>5.2819444444444441</v>
       </c>
@@ -905,7 +1072,7 @@
         <v>7.930555555555556E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>5.4683333333333337</v>
       </c>
@@ -922,7 +1089,7 @@
         <v>9.3194444444444441E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>5.5525000000000002</v>
       </c>
@@ -939,7 +1106,7 @@
         <v>4.2083333333333327E-2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>5.9474999999999998</v>
       </c>
@@ -956,7 +1123,7 @@
         <v>0.19750000000000001</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>6.1969444444444441</v>
       </c>
@@ -973,7 +1140,7 @@
         <v>0.12472222222222221</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>6.2616666666666667</v>
       </c>
@@ -990,7 +1157,7 @@
         <v>3.2361111111111111E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>6.7538888888888886</v>
       </c>
@@ -1007,7 +1174,7 @@
         <v>0.24611111111111111</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>7.2405555555555559</v>
       </c>
@@ -1024,7 +1191,7 @@
         <v>0.24333333333333329</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>7.3311111111111114</v>
       </c>
@@ -1041,7 +1208,7 @@
         <v>4.5277777777777778E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>7.5966666666666667</v>
       </c>
@@ -1058,7 +1225,7 @@
         <v>0.1327777777777778</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>7.7844444444444445</v>
       </c>
@@ -1075,7 +1242,7 @@
         <v>9.3888888888888883E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>8.586666666666666</v>
       </c>
@@ -1092,7 +1259,7 @@
         <v>0.40111111111111108</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>8.588055555555556</v>
       </c>
@@ -1109,7 +1276,7 @@
         <v>6.9444444444444447E-4</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>8.6333333333333329</v>
       </c>
@@ -1126,7 +1293,7 @@
         <v>2.2638888888888889E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>8.9474999999999998</v>
       </c>
@@ -1143,7 +1310,7 @@
         <v>0.1570833333333333</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>9.6894444444444439</v>
       </c>
@@ -1160,7 +1327,7 @@
         <v>0.3709722222222222</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>9.8291666666666675</v>
       </c>
@@ -1177,7 +1344,7 @@
         <v>6.986111111111111E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>10.000833333333333</v>
       </c>
@@ -1194,7 +1361,7 @@
         <v>8.5833333333333331E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>10.340833333333334</v>
       </c>
@@ -1211,7 +1378,7 @@
         <v>0.17</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>10.473611111111111</v>
       </c>
@@ -1228,7 +1395,7 @@
         <v>6.6388888888888886E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>10.755277777777778</v>
       </c>
@@ -1245,7 +1412,7 @@
         <v>0.14083333333333331</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>12.111388888888889</v>
       </c>
@@ -1262,7 +1429,7 @@
         <v>0.67805555555555552</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>12.328333333333333</v>
       </c>
@@ -1279,7 +1446,7 @@
         <v>0.10847222222222221</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>12.383333333333333</v>
       </c>
@@ -1296,7 +1463,7 @@
         <v>2.75E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>12.834722222222222</v>
       </c>
@@ -1313,7 +1480,7 @@
         <v>0.22569444444444439</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>13.064722222222223</v>
       </c>
@@ -1330,7 +1497,7 @@
         <v>0.115</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>14.023333333333333</v>
       </c>
@@ -1347,7 +1514,7 @@
         <v>0.47930555555555548</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>14.66611111111111</v>
       </c>
@@ -1364,7 +1531,7 @@
         <v>0.32138888888888889</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>14.934722222222222</v>
       </c>
@@ -1381,7 +1548,7 @@
         <v>0.13430555555555559</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>15.553888888888888</v>
       </c>
@@ -1398,7 +1565,7 @@
         <v>0.30958333333333332</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>16.003888888888888</v>
       </c>
@@ -1415,7 +1582,7 @@
         <v>0.22500000000000001</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>16.173888888888889</v>
       </c>
@@ -1432,7 +1599,7 @@
         <v>8.5000000000000006E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>16.322777777777777</v>
       </c>
@@ -1449,7 +1616,7 @@
         <v>7.4444444444444438E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>16.503055555555555</v>
       </c>
@@ -1466,7 +1633,7 @@
         <v>9.0138888888888893E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>17.040555555555557</v>
       </c>
@@ -1483,7 +1650,7 @@
         <v>0.26874999999999999</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>17.066388888888888</v>
       </c>
@@ -1500,7 +1667,7 @@
         <v>1.291666666666667E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>17.928333333333335</v>
       </c>
@@ -1519,6 +1686,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>